<commit_message>
Update Excel for TP2
Co-Authored-By: BURBECK-Heather-b24015232 <184231646+b24015232@users.noreply.github.com>
Co-Authored-By: ambreROFFIDAL <191879747+ambreROFFIDAL@users.noreply.github.com>
Co-Authored-By: ACHsofia <sofia.ach@etu.univ-amu.fr>
</commit_message>
<xml_diff>
--- a/TP_mesures_dev_web.xlsx
+++ b/TP_mesures_dev_web.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sofia\Documents\IUT\BUT3\ACH-ARFI-BURBECK-mesures\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/1c1c64e65d6dd269/Bureau/BUT Info/ACH-ARFI-BURBECK-ROFFIDAL-mesures/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{240C5AD3-9E77-4012-B467-BE16BC3F910B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="3" documentId="8_{240C5AD3-9E77-4012-B467-BE16BC3F910B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4D22293F-8B0D-48C7-9B6E-0B042B0BDB14}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="2" activeTab="10" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="LOC" sheetId="1" r:id="rId1"/>
@@ -22,6 +22,8 @@
     <sheet name="UFC devWeb" sheetId="9" r:id="rId7"/>
     <sheet name="Couplage" sheetId="11" r:id="rId8"/>
     <sheet name="Réponses" sheetId="12" r:id="rId9"/>
+    <sheet name="HPC Green Algorithms" sheetId="14" r:id="rId10"/>
+    <sheet name="EcoIndex" sheetId="15" r:id="rId11"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -44,7 +46,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="190" uniqueCount="159">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="250" uniqueCount="216">
   <si>
     <t>Lignes de code</t>
   </si>
@@ -540,6 +542,190 @@
   <si>
     <t>UFC QuickSort (illustration)</t>
   </si>
+  <si>
+    <t>C</t>
+  </si>
+  <si>
+    <t>t</t>
+  </si>
+  <si>
+    <t>Nom processeur</t>
+  </si>
+  <si>
+    <t>CPU ou GPU</t>
+  </si>
+  <si>
+    <t>n_p</t>
+  </si>
+  <si>
+    <t>n_c_p</t>
+  </si>
+  <si>
+    <t>n_c</t>
+  </si>
+  <si>
+    <t>TDP</t>
+  </si>
+  <si>
+    <t>P_c</t>
+  </si>
+  <si>
+    <t>u_c</t>
+  </si>
+  <si>
+    <t>mem/coeur 
+(jsp ce que c'est mais 
+normalement osef</t>
+  </si>
+  <si>
+    <t>n_m</t>
+  </si>
+  <si>
+    <t>P_m</t>
+  </si>
+  <si>
+    <t>PUE</t>
+  </si>
+  <si>
+    <t>CI</t>
+  </si>
+  <si>
+    <t>PSF</t>
+  </si>
+  <si>
+    <t>Sujet :</t>
+  </si>
+  <si>
+    <t>Xeon E5 2620</t>
+  </si>
+  <si>
+    <t>CPU</t>
+  </si>
+  <si>
+    <t>Légende :</t>
+  </si>
+  <si>
+    <t>C = Empreinte carbone (gCO2e (=grammes de gaz à effet de serre))</t>
+  </si>
+  <si>
+    <t>E = Consommation d'énergie (kWh)</t>
+  </si>
+  <si>
+    <t>t = temps d'exécution (h)</t>
+  </si>
+  <si>
+    <t>n_p = nombre de processeurs</t>
+  </si>
+  <si>
+    <t>n_c_p = nombre de coeurs par processeur</t>
+  </si>
+  <si>
+    <t>n_c = nombre total de coeurs (=n_p*n_c_p)</t>
+  </si>
+  <si>
+    <t>TDP = "Puissance de Dissipation Thermique" (W)</t>
+  </si>
+  <si>
+    <t>P_c = Puissance par Coeur (W) (=TDP/n_c_p)</t>
+  </si>
+  <si>
+    <t>u_c = facteur d'utilisation du processeur (entre 0 et 1 avec 1 = 100%)</t>
+  </si>
+  <si>
+    <t>n_m = mémoire disponible (Go)</t>
+  </si>
+  <si>
+    <t>P_m = Puissance consommée par la mémoire (W) (défaut=0,3725)</t>
+  </si>
+  <si>
+    <t>PUE = coefficient d'efficacité (défaut=1,67)</t>
+  </si>
+  <si>
+    <t>CI = Intensité Carbone de la production (défaut=475)</t>
+  </si>
+  <si>
+    <t>PSF = Facteur d'échelle pragmatique (défaut=1)</t>
+  </si>
+  <si>
+    <t>Les notations en jaune sont tirées du cours,
+les autres sont des nommages arbitraires</t>
+  </si>
+  <si>
+    <t>Les notations en vert dans le tableau sont des calculs auto.
+Pour le reste faut chercher dans la consigne et 
+les specs du processeur pour remplir le tableau</t>
+  </si>
+  <si>
+    <t>A calculer :</t>
+  </si>
+  <si>
+    <t>DOM : nombre d'éléments du DOM (noeuds)</t>
+  </si>
+  <si>
+    <t>Ko : données passant par le réseau entre client-serveur (en Ko)</t>
+  </si>
+  <si>
+    <t>HTTP : nombre de requêtes HTTP</t>
+  </si>
+  <si>
+    <t>Avec ces éléments, utilisez le tableau suivant (calcul auto) :</t>
+  </si>
+  <si>
+    <t>DOM</t>
+  </si>
+  <si>
+    <t>Quantile</t>
+  </si>
+  <si>
+    <t>Quantile(xDOM)</t>
+  </si>
+  <si>
+    <t>Ko</t>
+  </si>
+  <si>
+    <t>Quantile (xKo)</t>
+  </si>
+  <si>
+    <t>HTTP</t>
+  </si>
+  <si>
+    <t>Quantile (xHTTP)</t>
+  </si>
+  <si>
+    <t>nomdusite.com</t>
+  </si>
+  <si>
+    <t>Pour les quantiles, voir le tableau suivant :</t>
+  </si>
+  <si>
+    <t>Quantile (n)</t>
+  </si>
+  <si>
+    <t>Borne
+DOM</t>
+  </si>
+  <si>
+    <t>Borne
+Ko</t>
+  </si>
+  <si>
+    <t>Borne
+HTTP</t>
+  </si>
+  <si>
+    <t>Arbitraire : 
+aide au 
+calcul auto</t>
+  </si>
+  <si>
+    <t>Resultat 
+EcoIndex
+arrondi</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Résultat 
+EcoIndex </t>
+  </si>
 </sst>
 </file>
 
@@ -551,7 +737,7 @@
     <numFmt numFmtId="166" formatCode="_(\$* #,##0.00_);_(\$* \(#,##0.00\);_(\$* \-??_);_(@_)"/>
     <numFmt numFmtId="167" formatCode="_(\$* #,##0_);_(\$* \(#,##0\);_(\$* \-_);_(@_)"/>
   </numFmts>
-  <fonts count="5">
+  <fonts count="8">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -580,16 +766,47 @@
       <sz val="10"/>
       <name val="Arial Unicode MS"/>
     </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="10"/>
+      <color theme="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <charset val="1"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFB6D7A8"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="12">
     <border>
       <left/>
       <right/>
@@ -597,16 +814,166 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color rgb="FFCCCCCC"/>
+      </left>
+      <right style="medium">
+        <color rgb="FFCCCCCC"/>
+      </right>
+      <top style="medium">
+        <color rgb="FFCCCCCC"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FFCCCCCC"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FFCCCCCC"/>
+      </left>
+      <right/>
+      <top style="medium">
+        <color rgb="FFCCCCCC"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FFCCCCCC"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color rgb="FFCCCCCC"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FFCCCCCC"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color rgb="FFCCCCCC"/>
+      </right>
+      <top style="medium">
+        <color rgb="FFCCCCCC"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FFCCCCCC"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FFCCCCCC"/>
+      </left>
+      <right style="medium">
+        <color rgb="FFCCCCCC"/>
+      </right>
+      <top style="medium">
+        <color rgb="FFCCCCCC"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="medium">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="medium">
+        <color rgb="FFCCCCCC"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FFCCCCCC"/>
+      </left>
+      <right style="medium">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="medium">
+        <color rgb="FFCCCCCC"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="medium">
+        <color rgb="FF000000"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF000000"/>
+      </left>
+      <right/>
+      <top style="medium">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="medium">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="medium">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="medium">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="6">
+  <cellStyleXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="164" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="165" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="166" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="167" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="33">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -626,12 +993,85 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="4" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="6" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="6">
+  <cellStyles count="7">
     <cellStyle name="Comma" xfId="1" xr:uid="{00000000-0005-0000-0000-000006000000}"/>
     <cellStyle name="Comma [0]" xfId="2" xr:uid="{00000000-0005-0000-0000-000007000000}"/>
     <cellStyle name="Currency" xfId="3" xr:uid="{00000000-0005-0000-0000-000008000000}"/>
     <cellStyle name="Currency [0]" xfId="4" xr:uid="{00000000-0005-0000-0000-000009000000}"/>
+    <cellStyle name="Lien hypertexte" xfId="6" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Percent" xfId="5" xr:uid="{00000000-0005-0000-0000-00000A000000}"/>
   </cellStyles>
@@ -646,6 +1086,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -815,6 +1259,1399 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FC84E6A1-3985-496B-B8E9-FF7B55C63621}">
+  <dimension ref="A1:R22"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="13.2"/>
+  <cols>
+    <col min="1" max="1" width="58.88671875" customWidth="1"/>
+    <col min="6" max="6" width="15.33203125" customWidth="1"/>
+    <col min="8" max="8" width="12.77734375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:18" ht="13.8" thickBot="1">
+      <c r="A1" s="9"/>
+      <c r="B1" s="9"/>
+      <c r="C1" s="9"/>
+      <c r="D1" s="9"/>
+      <c r="E1" s="9"/>
+      <c r="F1" s="9"/>
+      <c r="G1" s="9"/>
+      <c r="H1" s="9"/>
+      <c r="I1" s="9"/>
+      <c r="J1" s="9"/>
+      <c r="K1" s="9"/>
+      <c r="L1" s="9"/>
+      <c r="M1" s="9"/>
+      <c r="N1" s="9"/>
+      <c r="O1" s="9"/>
+      <c r="P1" s="9"/>
+      <c r="Q1" s="9"/>
+      <c r="R1" s="9"/>
+    </row>
+    <row r="2" spans="1:18" ht="66.599999999999994" thickBot="1">
+      <c r="A2" s="9"/>
+      <c r="B2" s="10" t="s">
+        <v>159</v>
+      </c>
+      <c r="C2" s="10" t="s">
+        <v>10</v>
+      </c>
+      <c r="D2" s="9" t="s">
+        <v>160</v>
+      </c>
+      <c r="E2" s="9" t="s">
+        <v>161</v>
+      </c>
+      <c r="F2" s="9" t="s">
+        <v>162</v>
+      </c>
+      <c r="G2" s="9" t="s">
+        <v>163</v>
+      </c>
+      <c r="H2" s="9" t="s">
+        <v>164</v>
+      </c>
+      <c r="I2" s="10" t="s">
+        <v>165</v>
+      </c>
+      <c r="J2" s="9" t="s">
+        <v>166</v>
+      </c>
+      <c r="K2" s="10" t="s">
+        <v>167</v>
+      </c>
+      <c r="L2" s="9" t="s">
+        <v>168</v>
+      </c>
+      <c r="M2" s="9" t="s">
+        <v>169</v>
+      </c>
+      <c r="N2" s="9" t="s">
+        <v>170</v>
+      </c>
+      <c r="O2" s="9" t="s">
+        <v>171</v>
+      </c>
+      <c r="P2" s="9" t="s">
+        <v>172</v>
+      </c>
+      <c r="Q2" s="9" t="s">
+        <v>173</v>
+      </c>
+      <c r="R2" s="9" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="3" spans="1:18" ht="27" thickBot="1">
+      <c r="A3" s="9" t="s">
+        <v>175</v>
+      </c>
+      <c r="B3" s="11">
+        <f>ROUND(C3*Q3, 0)</f>
+        <v>53463</v>
+      </c>
+      <c r="C3" s="11">
+        <f>(D3*((I3*K3*L3)+(N3*O3))*P3*R3*0.001)</f>
+        <v>112.55365799999998</v>
+      </c>
+      <c r="D3" s="12">
+        <v>504</v>
+      </c>
+      <c r="E3" s="9" t="s">
+        <v>176</v>
+      </c>
+      <c r="F3" s="9" t="s">
+        <v>177</v>
+      </c>
+      <c r="G3" s="12">
+        <v>1</v>
+      </c>
+      <c r="H3" s="12">
+        <v>12</v>
+      </c>
+      <c r="I3" s="11">
+        <f>H3*G3</f>
+        <v>12</v>
+      </c>
+      <c r="J3" s="12">
+        <v>130</v>
+      </c>
+      <c r="K3" s="11">
+        <f>J3/I3</f>
+        <v>10.833333333333334</v>
+      </c>
+      <c r="L3" s="12">
+        <v>1</v>
+      </c>
+      <c r="M3" s="9"/>
+      <c r="N3" s="12">
+        <v>10</v>
+      </c>
+      <c r="O3" s="12">
+        <v>0.3725</v>
+      </c>
+      <c r="P3" s="12">
+        <v>1.67</v>
+      </c>
+      <c r="Q3" s="12">
+        <v>475</v>
+      </c>
+      <c r="R3" s="12">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:18" ht="13.8" thickBot="1">
+      <c r="A4" s="9"/>
+      <c r="B4" s="9"/>
+      <c r="C4" s="9"/>
+      <c r="D4" s="9"/>
+      <c r="E4" s="9"/>
+      <c r="F4" s="9"/>
+      <c r="G4" s="9"/>
+      <c r="H4" s="9"/>
+      <c r="I4" s="9"/>
+      <c r="J4" s="9"/>
+      <c r="K4" s="9"/>
+      <c r="L4" s="9"/>
+      <c r="M4" s="9"/>
+      <c r="N4" s="9"/>
+      <c r="O4" s="9"/>
+      <c r="P4" s="9"/>
+      <c r="Q4" s="9"/>
+      <c r="R4" s="9"/>
+    </row>
+    <row r="5" spans="1:18" ht="13.8" thickBot="1">
+      <c r="A5" s="9"/>
+      <c r="B5" s="9"/>
+      <c r="C5" s="9"/>
+      <c r="D5" s="9"/>
+      <c r="E5" s="9"/>
+      <c r="F5" s="9"/>
+      <c r="G5" s="9"/>
+      <c r="H5" s="9"/>
+      <c r="I5" s="9"/>
+      <c r="J5" s="9"/>
+      <c r="K5" s="9"/>
+      <c r="L5" s="9"/>
+      <c r="M5" s="9"/>
+      <c r="N5" s="9"/>
+      <c r="O5" s="9"/>
+      <c r="P5" s="9"/>
+      <c r="Q5" s="9"/>
+      <c r="R5" s="9"/>
+    </row>
+    <row r="6" spans="1:18" ht="15.6" customHeight="1" thickBot="1">
+      <c r="A6" s="9"/>
+      <c r="B6" s="9"/>
+      <c r="C6" s="9"/>
+      <c r="D6" s="9"/>
+      <c r="E6" s="9"/>
+      <c r="F6" s="9"/>
+      <c r="G6" s="9"/>
+      <c r="H6" s="9"/>
+      <c r="I6" s="9"/>
+      <c r="J6" s="9"/>
+      <c r="K6" s="9"/>
+      <c r="L6" s="9"/>
+      <c r="M6" s="9"/>
+      <c r="N6" s="9"/>
+      <c r="O6" s="9"/>
+      <c r="P6" s="9"/>
+      <c r="Q6" s="9"/>
+      <c r="R6" s="9"/>
+    </row>
+    <row r="7" spans="1:18" ht="43.2" customHeight="1" thickBot="1">
+      <c r="A7" s="9" t="s">
+        <v>178</v>
+      </c>
+      <c r="B7" s="9"/>
+      <c r="C7" s="9"/>
+      <c r="D7" s="9"/>
+      <c r="E7" s="9"/>
+      <c r="F7" s="28" t="s">
+        <v>193</v>
+      </c>
+      <c r="G7" s="29"/>
+      <c r="H7" s="30"/>
+      <c r="I7" s="9"/>
+      <c r="J7" s="9"/>
+      <c r="K7" s="9"/>
+      <c r="L7" s="9"/>
+      <c r="M7" s="9"/>
+      <c r="N7" s="9"/>
+      <c r="O7" s="9"/>
+      <c r="P7" s="9"/>
+      <c r="Q7" s="9"/>
+      <c r="R7" s="9"/>
+    </row>
+    <row r="8" spans="1:18" ht="56.4" customHeight="1" thickBot="1">
+      <c r="A8" s="14" t="s">
+        <v>179</v>
+      </c>
+      <c r="B8" s="9"/>
+      <c r="C8" s="9"/>
+      <c r="D8" s="9"/>
+      <c r="E8" s="9"/>
+      <c r="F8" s="28" t="s">
+        <v>194</v>
+      </c>
+      <c r="G8" s="31"/>
+      <c r="H8" s="32"/>
+      <c r="I8" s="9"/>
+      <c r="J8" s="9"/>
+      <c r="K8" s="9"/>
+      <c r="L8" s="9"/>
+      <c r="M8" s="9"/>
+      <c r="N8" s="9"/>
+      <c r="O8" s="9"/>
+      <c r="P8" s="9"/>
+      <c r="Q8" s="9"/>
+      <c r="R8" s="9"/>
+    </row>
+    <row r="9" spans="1:18" ht="13.8" thickBot="1">
+      <c r="A9" s="14" t="s">
+        <v>180</v>
+      </c>
+      <c r="B9" s="9"/>
+      <c r="C9" s="9"/>
+      <c r="D9" s="9"/>
+      <c r="E9" s="9"/>
+      <c r="F9" s="9"/>
+      <c r="G9" s="9"/>
+      <c r="H9" s="9"/>
+      <c r="I9" s="9"/>
+      <c r="J9" s="9"/>
+      <c r="K9" s="9"/>
+      <c r="L9" s="9"/>
+      <c r="M9" s="9"/>
+      <c r="N9" s="9"/>
+      <c r="O9" s="9"/>
+      <c r="P9" s="9"/>
+      <c r="Q9" s="9"/>
+      <c r="R9" s="9"/>
+    </row>
+    <row r="10" spans="1:18" ht="13.8" thickBot="1">
+      <c r="A10" s="14" t="s">
+        <v>181</v>
+      </c>
+      <c r="B10" s="9"/>
+      <c r="C10" s="9"/>
+      <c r="D10" s="9"/>
+      <c r="E10" s="9"/>
+      <c r="F10" s="9"/>
+      <c r="G10" s="9"/>
+      <c r="H10" s="9"/>
+      <c r="I10" s="9"/>
+      <c r="J10" s="9"/>
+      <c r="K10" s="9"/>
+      <c r="L10" s="9"/>
+      <c r="M10" s="9"/>
+      <c r="N10" s="9"/>
+      <c r="O10" s="9"/>
+      <c r="P10" s="9"/>
+      <c r="Q10" s="9"/>
+      <c r="R10" s="9"/>
+    </row>
+    <row r="11" spans="1:18" ht="13.8" thickBot="1">
+      <c r="A11" s="9" t="s">
+        <v>182</v>
+      </c>
+      <c r="B11" s="9"/>
+      <c r="C11" s="9"/>
+      <c r="D11" s="9"/>
+      <c r="E11" s="9"/>
+      <c r="F11" s="9"/>
+      <c r="G11" s="9"/>
+      <c r="H11" s="9"/>
+      <c r="I11" s="9"/>
+      <c r="J11" s="9"/>
+      <c r="K11" s="9"/>
+      <c r="L11" s="9"/>
+      <c r="M11" s="9"/>
+      <c r="N11" s="9"/>
+      <c r="O11" s="9"/>
+      <c r="P11" s="9"/>
+      <c r="Q11" s="9"/>
+      <c r="R11" s="9"/>
+    </row>
+    <row r="12" spans="1:18" ht="13.8" thickBot="1">
+      <c r="A12" s="9" t="s">
+        <v>183</v>
+      </c>
+      <c r="B12" s="9"/>
+      <c r="C12" s="9"/>
+      <c r="D12" s="9"/>
+      <c r="E12" s="9"/>
+      <c r="F12" s="9"/>
+      <c r="G12" s="9"/>
+      <c r="H12" s="9"/>
+      <c r="I12" s="9"/>
+      <c r="J12" s="9"/>
+      <c r="K12" s="9"/>
+      <c r="L12" s="9"/>
+      <c r="M12" s="9"/>
+      <c r="N12" s="9"/>
+      <c r="O12" s="9"/>
+      <c r="P12" s="9"/>
+      <c r="Q12" s="9"/>
+      <c r="R12" s="9"/>
+    </row>
+    <row r="13" spans="1:18" ht="13.8" thickBot="1">
+      <c r="A13" s="14" t="s">
+        <v>184</v>
+      </c>
+      <c r="B13" s="9"/>
+      <c r="C13" s="9"/>
+      <c r="D13" s="9"/>
+      <c r="E13" s="9"/>
+      <c r="F13" s="9"/>
+      <c r="G13" s="9"/>
+      <c r="H13" s="9"/>
+      <c r="I13" s="9"/>
+      <c r="J13" s="9"/>
+      <c r="K13" s="9"/>
+      <c r="L13" s="9"/>
+      <c r="M13" s="9"/>
+      <c r="N13" s="9"/>
+      <c r="O13" s="9"/>
+      <c r="P13" s="9"/>
+      <c r="Q13" s="9"/>
+      <c r="R13" s="9"/>
+    </row>
+    <row r="14" spans="1:18" ht="13.8" thickBot="1">
+      <c r="A14" s="14" t="s">
+        <v>185</v>
+      </c>
+      <c r="B14" s="9"/>
+      <c r="C14" s="9"/>
+      <c r="D14" s="9"/>
+      <c r="E14" s="9"/>
+      <c r="F14" s="9"/>
+      <c r="G14" s="9"/>
+      <c r="H14" s="9"/>
+      <c r="I14" s="9"/>
+      <c r="J14" s="9"/>
+      <c r="K14" s="9"/>
+      <c r="L14" s="9"/>
+      <c r="M14" s="9"/>
+      <c r="N14" s="9"/>
+      <c r="O14" s="9"/>
+      <c r="P14" s="9"/>
+      <c r="Q14" s="9"/>
+      <c r="R14" s="9"/>
+    </row>
+    <row r="15" spans="1:18" ht="13.8" thickBot="1">
+      <c r="A15" s="14" t="s">
+        <v>186</v>
+      </c>
+      <c r="B15" s="9"/>
+      <c r="C15" s="9"/>
+      <c r="D15" s="9"/>
+      <c r="E15" s="9"/>
+      <c r="F15" s="9"/>
+      <c r="G15" s="9"/>
+      <c r="H15" s="9"/>
+      <c r="I15" s="9"/>
+      <c r="J15" s="9"/>
+      <c r="K15" s="9"/>
+      <c r="L15" s="9"/>
+      <c r="M15" s="9"/>
+      <c r="N15" s="9"/>
+      <c r="O15" s="9"/>
+      <c r="P15" s="9"/>
+      <c r="Q15" s="9"/>
+      <c r="R15" s="9"/>
+    </row>
+    <row r="16" spans="1:18" ht="13.8" thickBot="1">
+      <c r="A16" s="14" t="s">
+        <v>187</v>
+      </c>
+      <c r="B16" s="9"/>
+      <c r="C16" s="9"/>
+      <c r="D16" s="9"/>
+      <c r="E16" s="9"/>
+      <c r="F16" s="9"/>
+      <c r="G16" s="9"/>
+      <c r="H16" s="9"/>
+      <c r="I16" s="9"/>
+      <c r="J16" s="9"/>
+      <c r="K16" s="9"/>
+      <c r="L16" s="9"/>
+      <c r="M16" s="9"/>
+      <c r="N16" s="9"/>
+      <c r="O16" s="9"/>
+      <c r="P16" s="9"/>
+      <c r="Q16" s="9"/>
+      <c r="R16" s="9"/>
+    </row>
+    <row r="17" spans="1:18" ht="13.8" thickBot="1">
+      <c r="A17" s="14" t="s">
+        <v>188</v>
+      </c>
+      <c r="B17" s="9"/>
+      <c r="C17" s="9"/>
+      <c r="D17" s="9"/>
+      <c r="E17" s="9"/>
+      <c r="F17" s="9"/>
+      <c r="G17" s="9"/>
+      <c r="H17" s="9"/>
+      <c r="I17" s="9"/>
+      <c r="J17" s="9"/>
+      <c r="K17" s="9"/>
+      <c r="L17" s="9"/>
+      <c r="M17" s="9"/>
+      <c r="N17" s="9"/>
+      <c r="O17" s="9"/>
+      <c r="P17" s="9"/>
+      <c r="Q17" s="9"/>
+      <c r="R17" s="9"/>
+    </row>
+    <row r="18" spans="1:18" ht="13.8" thickBot="1">
+      <c r="A18" s="14" t="s">
+        <v>189</v>
+      </c>
+      <c r="B18" s="9"/>
+      <c r="C18" s="9"/>
+      <c r="D18" s="9"/>
+      <c r="E18" s="9"/>
+      <c r="F18" s="9"/>
+      <c r="G18" s="9"/>
+      <c r="H18" s="9"/>
+      <c r="I18" s="9"/>
+      <c r="J18" s="9"/>
+      <c r="K18" s="9"/>
+      <c r="L18" s="9"/>
+      <c r="M18" s="9"/>
+      <c r="N18" s="9"/>
+      <c r="O18" s="9"/>
+      <c r="P18" s="9"/>
+      <c r="Q18" s="9"/>
+      <c r="R18" s="9"/>
+    </row>
+    <row r="19" spans="1:18" ht="13.8" thickBot="1">
+      <c r="A19" s="14" t="s">
+        <v>190</v>
+      </c>
+      <c r="B19" s="9"/>
+      <c r="C19" s="9"/>
+      <c r="D19" s="9"/>
+      <c r="E19" s="9"/>
+      <c r="F19" s="9"/>
+      <c r="G19" s="9"/>
+      <c r="H19" s="9"/>
+      <c r="I19" s="9"/>
+      <c r="J19" s="9"/>
+      <c r="K19" s="9"/>
+      <c r="L19" s="9"/>
+      <c r="M19" s="9"/>
+      <c r="N19" s="9"/>
+      <c r="O19" s="9"/>
+      <c r="P19" s="9"/>
+      <c r="Q19" s="9"/>
+      <c r="R19" s="9"/>
+    </row>
+    <row r="20" spans="1:18" ht="13.8" thickBot="1">
+      <c r="A20" s="14" t="s">
+        <v>191</v>
+      </c>
+      <c r="B20" s="9"/>
+      <c r="C20" s="9"/>
+      <c r="D20" s="9"/>
+      <c r="E20" s="9"/>
+      <c r="F20" s="9"/>
+      <c r="G20" s="9"/>
+      <c r="H20" s="9"/>
+      <c r="I20" s="9"/>
+      <c r="J20" s="9"/>
+      <c r="K20" s="9"/>
+      <c r="L20" s="9"/>
+      <c r="M20" s="9"/>
+      <c r="N20" s="9"/>
+      <c r="O20" s="9"/>
+      <c r="P20" s="9"/>
+      <c r="Q20" s="9"/>
+      <c r="R20" s="9"/>
+    </row>
+    <row r="21" spans="1:18" ht="13.8" thickBot="1">
+      <c r="A21" s="14" t="s">
+        <v>192</v>
+      </c>
+      <c r="B21" s="9"/>
+      <c r="C21" s="9"/>
+      <c r="D21" s="9"/>
+      <c r="E21" s="9"/>
+      <c r="F21" s="9"/>
+      <c r="G21" s="9"/>
+      <c r="H21" s="9"/>
+      <c r="I21" s="9"/>
+      <c r="J21" s="9"/>
+      <c r="K21" s="9"/>
+      <c r="L21" s="9"/>
+      <c r="M21" s="9"/>
+      <c r="N21" s="9"/>
+      <c r="O21" s="9"/>
+      <c r="P21" s="9"/>
+      <c r="Q21" s="9"/>
+      <c r="R21" s="9"/>
+    </row>
+    <row r="22" spans="1:18" ht="13.8" thickBot="1">
+      <c r="A22" s="9"/>
+      <c r="B22" s="9"/>
+      <c r="C22" s="9"/>
+      <c r="D22" s="9"/>
+      <c r="E22" s="9"/>
+      <c r="F22" s="9"/>
+      <c r="G22" s="9"/>
+      <c r="H22" s="9"/>
+      <c r="I22" s="9"/>
+      <c r="J22" s="9"/>
+      <c r="K22" s="9"/>
+      <c r="L22" s="9"/>
+      <c r="M22" s="9"/>
+      <c r="N22" s="9"/>
+      <c r="O22" s="9"/>
+      <c r="P22" s="9"/>
+      <c r="Q22" s="9"/>
+      <c r="R22" s="9"/>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="F7:H7"/>
+    <mergeCell ref="F8:H8"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7693CCEA-4A50-434C-8CF1-1DBFE0F7E32A}">
+  <dimension ref="A1:L36"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="13.2"/>
+  <sheetData>
+    <row r="1" spans="1:12" ht="13.8" thickBot="1">
+      <c r="A1" s="9" t="s">
+        <v>195</v>
+      </c>
+      <c r="B1" s="9"/>
+      <c r="C1" s="9"/>
+      <c r="D1" s="9"/>
+      <c r="E1" s="9"/>
+      <c r="F1" s="9"/>
+      <c r="G1" s="9"/>
+      <c r="H1" s="9"/>
+      <c r="I1" s="9"/>
+      <c r="J1" s="9"/>
+      <c r="K1" s="9"/>
+      <c r="L1" s="9"/>
+    </row>
+    <row r="2" spans="1:12" ht="13.8" thickBot="1">
+      <c r="A2" s="13" t="s">
+        <v>196</v>
+      </c>
+      <c r="B2" s="9"/>
+      <c r="C2" s="9"/>
+      <c r="D2" s="9"/>
+      <c r="E2" s="9"/>
+      <c r="F2" s="9"/>
+      <c r="G2" s="9"/>
+      <c r="H2" s="9"/>
+      <c r="I2" s="9"/>
+      <c r="J2" s="9"/>
+      <c r="K2" s="9"/>
+      <c r="L2" s="9"/>
+    </row>
+    <row r="3" spans="1:12" ht="13.8" thickBot="1">
+      <c r="A3" s="13" t="s">
+        <v>197</v>
+      </c>
+      <c r="B3" s="9"/>
+      <c r="C3" s="9"/>
+      <c r="D3" s="9"/>
+      <c r="E3" s="9"/>
+      <c r="F3" s="9"/>
+      <c r="G3" s="9"/>
+      <c r="H3" s="9"/>
+      <c r="I3" s="9"/>
+      <c r="J3" s="9"/>
+      <c r="K3" s="9"/>
+      <c r="L3" s="9"/>
+    </row>
+    <row r="4" spans="1:12" ht="13.8" thickBot="1">
+      <c r="A4" s="13" t="s">
+        <v>198</v>
+      </c>
+      <c r="B4" s="9"/>
+      <c r="C4" s="9"/>
+      <c r="D4" s="9"/>
+      <c r="E4" s="9"/>
+      <c r="F4" s="9"/>
+      <c r="G4" s="9"/>
+      <c r="H4" s="9"/>
+      <c r="I4" s="13"/>
+      <c r="J4" s="9"/>
+      <c r="K4" s="9"/>
+      <c r="L4" s="9"/>
+    </row>
+    <row r="5" spans="1:12" ht="13.8" thickBot="1">
+      <c r="A5" s="9"/>
+      <c r="B5" s="9"/>
+      <c r="C5" s="9"/>
+      <c r="D5" s="9"/>
+      <c r="E5" s="9"/>
+      <c r="F5" s="9"/>
+      <c r="G5" s="9"/>
+      <c r="H5" s="9"/>
+      <c r="I5" s="13"/>
+      <c r="J5" s="9"/>
+      <c r="K5" s="9"/>
+      <c r="L5" s="9"/>
+    </row>
+    <row r="6" spans="1:12" ht="13.8" thickBot="1">
+      <c r="A6" s="13" t="s">
+        <v>199</v>
+      </c>
+      <c r="B6" s="9"/>
+      <c r="C6" s="9"/>
+      <c r="D6" s="9"/>
+      <c r="E6" s="9"/>
+      <c r="F6" s="9"/>
+      <c r="G6" s="9"/>
+      <c r="H6" s="9"/>
+      <c r="I6" s="9"/>
+      <c r="J6" s="9"/>
+      <c r="K6" s="9"/>
+      <c r="L6" s="9"/>
+    </row>
+    <row r="7" spans="1:12" ht="13.8" thickBot="1">
+      <c r="A7" s="9"/>
+      <c r="B7" s="9"/>
+      <c r="C7" s="9"/>
+      <c r="D7" s="9"/>
+      <c r="E7" s="9"/>
+      <c r="F7" s="9"/>
+      <c r="G7" s="9"/>
+      <c r="H7" s="9"/>
+      <c r="I7" s="9"/>
+      <c r="J7" s="9"/>
+      <c r="K7" s="9"/>
+      <c r="L7" s="9"/>
+    </row>
+    <row r="8" spans="1:12" ht="40.200000000000003" thickBot="1">
+      <c r="A8" s="9"/>
+      <c r="B8" s="9" t="s">
+        <v>214</v>
+      </c>
+      <c r="C8" s="9" t="s">
+        <v>215</v>
+      </c>
+      <c r="D8" s="14" t="s">
+        <v>200</v>
+      </c>
+      <c r="E8" s="9" t="s">
+        <v>201</v>
+      </c>
+      <c r="F8" s="9" t="s">
+        <v>202</v>
+      </c>
+      <c r="G8" s="14" t="s">
+        <v>203</v>
+      </c>
+      <c r="H8" s="9" t="s">
+        <v>201</v>
+      </c>
+      <c r="I8" s="9" t="s">
+        <v>204</v>
+      </c>
+      <c r="J8" s="14" t="s">
+        <v>205</v>
+      </c>
+      <c r="K8" s="9" t="s">
+        <v>201</v>
+      </c>
+      <c r="L8" s="9" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="9" spans="1:12" ht="27" thickBot="1">
+      <c r="A9" s="15" t="s">
+        <v>207</v>
+      </c>
+      <c r="B9" s="12">
+        <f>ROUND(C9, 0)</f>
+        <v>88</v>
+      </c>
+      <c r="C9" s="12">
+        <f>100-5*(3*F9+2*I9+L9)/6</f>
+        <v>88.054447574785257</v>
+      </c>
+      <c r="D9" s="16">
+        <v>205</v>
+      </c>
+      <c r="E9" s="12">
+        <f>INDEX(F15:F35, MATCH(D9, C15:C35, 1))</f>
+        <v>4</v>
+      </c>
+      <c r="F9" s="12">
+        <f>(E9 - 1) + (D9 - INDEX(C15:C35, E9)) / (INDEX(C15:C35, E9 + 1) - INDEX(C15:C35, E9))</f>
+        <v>3.6216216216216215</v>
+      </c>
+      <c r="G9" s="16">
+        <v>18.5</v>
+      </c>
+      <c r="H9" s="12">
+        <f>INDEX(F15:F35, MATCH(G9, D15:D35, 1))</f>
+        <v>2</v>
+      </c>
+      <c r="I9" s="12">
+        <f>(H9 - 1) + (G9 - INDEX(D15:D35, H9)) / (INDEX(D15:D35, H9 + 1) - INDEX(D15:D35, H9))</f>
+        <v>1.119514407311798</v>
+      </c>
+      <c r="J9" s="16">
+        <v>5</v>
+      </c>
+      <c r="K9" s="12">
+        <f>INDEX(F15:F35, MATCH(J9, E15:E35, 1))</f>
+        <v>2</v>
+      </c>
+      <c r="L9" s="12">
+        <f>(K9 - 1) + (J9 - INDEX(E15:E35, K9)) / (INDEX(E15:E35, K9 + 1) - INDEX(E15:E35, K9))</f>
+        <v>1.2307692307692308</v>
+      </c>
+    </row>
+    <row r="10" spans="1:12" ht="13.8" thickBot="1">
+      <c r="A10" s="9"/>
+      <c r="B10" s="9"/>
+      <c r="C10" s="9"/>
+      <c r="D10" s="9"/>
+      <c r="E10" s="9"/>
+      <c r="F10" s="9"/>
+      <c r="G10" s="9"/>
+      <c r="H10" s="9"/>
+      <c r="I10" s="9"/>
+      <c r="J10" s="9"/>
+      <c r="K10" s="9"/>
+      <c r="L10" s="9"/>
+    </row>
+    <row r="11" spans="1:12" ht="13.8" thickBot="1">
+      <c r="A11" s="9"/>
+      <c r="B11" s="9"/>
+      <c r="C11" s="9"/>
+      <c r="D11" s="9"/>
+      <c r="E11" s="9"/>
+      <c r="F11" s="9"/>
+      <c r="G11" s="9"/>
+      <c r="H11" s="9"/>
+      <c r="I11" s="9"/>
+      <c r="J11" s="9"/>
+      <c r="K11" s="9"/>
+      <c r="L11" s="9"/>
+    </row>
+    <row r="12" spans="1:12" ht="13.8" thickBot="1">
+      <c r="A12" s="13" t="s">
+        <v>208</v>
+      </c>
+      <c r="B12" s="9"/>
+      <c r="C12" s="9"/>
+      <c r="D12" s="9"/>
+      <c r="E12" s="9"/>
+      <c r="F12" s="9"/>
+      <c r="G12" s="9"/>
+      <c r="H12" s="9"/>
+      <c r="I12" s="9"/>
+      <c r="J12" s="9"/>
+      <c r="K12" s="9"/>
+      <c r="L12" s="9"/>
+    </row>
+    <row r="13" spans="1:12" ht="13.8" thickBot="1">
+      <c r="A13" s="17"/>
+      <c r="B13" s="17"/>
+      <c r="C13" s="17"/>
+      <c r="D13" s="17"/>
+      <c r="E13" s="17"/>
+      <c r="F13" s="17"/>
+      <c r="G13" s="9"/>
+      <c r="H13" s="9"/>
+      <c r="I13" s="9"/>
+      <c r="J13" s="9"/>
+      <c r="K13" s="9"/>
+      <c r="L13" s="9"/>
+    </row>
+    <row r="14" spans="1:12" ht="40.200000000000003" thickBot="1">
+      <c r="A14" s="26" t="s">
+        <v>209</v>
+      </c>
+      <c r="B14" s="27"/>
+      <c r="C14" s="18" t="s">
+        <v>210</v>
+      </c>
+      <c r="D14" s="18" t="s">
+        <v>211</v>
+      </c>
+      <c r="E14" s="18" t="s">
+        <v>212</v>
+      </c>
+      <c r="F14" s="18" t="s">
+        <v>213</v>
+      </c>
+      <c r="G14" s="9"/>
+      <c r="H14" s="9"/>
+      <c r="I14" s="9"/>
+      <c r="J14" s="9"/>
+      <c r="K14" s="9"/>
+      <c r="L14" s="9"/>
+    </row>
+    <row r="15" spans="1:12" ht="13.8" thickBot="1">
+      <c r="A15" s="19"/>
+      <c r="B15" s="24">
+        <v>1</v>
+      </c>
+      <c r="C15" s="20">
+        <v>0</v>
+      </c>
+      <c r="D15" s="20">
+        <v>0</v>
+      </c>
+      <c r="E15" s="20">
+        <v>0</v>
+      </c>
+      <c r="F15" s="21">
+        <v>1</v>
+      </c>
+      <c r="G15" s="9"/>
+      <c r="H15" s="9"/>
+      <c r="I15" s="9"/>
+      <c r="J15" s="9"/>
+      <c r="K15" s="9"/>
+      <c r="L15" s="9"/>
+    </row>
+    <row r="16" spans="1:12" ht="13.8" thickBot="1">
+      <c r="A16" s="24">
+        <v>2</v>
+      </c>
+      <c r="B16" s="25"/>
+      <c r="C16" s="20">
+        <v>47</v>
+      </c>
+      <c r="D16" s="20">
+        <v>1.37</v>
+      </c>
+      <c r="E16" s="20">
+        <v>2</v>
+      </c>
+      <c r="F16" s="21">
+        <v>2</v>
+      </c>
+      <c r="G16" s="9"/>
+      <c r="H16" s="9"/>
+      <c r="I16" s="9"/>
+      <c r="J16" s="9"/>
+      <c r="K16" s="9"/>
+      <c r="L16" s="9"/>
+    </row>
+    <row r="17" spans="1:12" ht="13.8" thickBot="1">
+      <c r="A17" s="25"/>
+      <c r="B17" s="24">
+        <v>3</v>
+      </c>
+      <c r="C17" s="20">
+        <v>75</v>
+      </c>
+      <c r="D17" s="20">
+        <v>144.69999999999999</v>
+      </c>
+      <c r="E17" s="20">
+        <v>15</v>
+      </c>
+      <c r="F17" s="21">
+        <v>3</v>
+      </c>
+      <c r="G17" s="9"/>
+      <c r="H17" s="9"/>
+      <c r="I17" s="9"/>
+      <c r="J17" s="9"/>
+      <c r="K17" s="9"/>
+      <c r="L17" s="9"/>
+    </row>
+    <row r="18" spans="1:12" ht="13.8" thickBot="1">
+      <c r="A18" s="24">
+        <v>4</v>
+      </c>
+      <c r="B18" s="25"/>
+      <c r="C18" s="20">
+        <v>159</v>
+      </c>
+      <c r="D18" s="20">
+        <v>319.52999999999997</v>
+      </c>
+      <c r="E18" s="20">
+        <v>25</v>
+      </c>
+      <c r="F18" s="21">
+        <v>4</v>
+      </c>
+      <c r="G18" s="9"/>
+      <c r="H18" s="9"/>
+      <c r="I18" s="9"/>
+      <c r="J18" s="9"/>
+      <c r="K18" s="9"/>
+      <c r="L18" s="9"/>
+    </row>
+    <row r="19" spans="1:12" ht="13.8" thickBot="1">
+      <c r="A19" s="25"/>
+      <c r="B19" s="24">
+        <v>5</v>
+      </c>
+      <c r="C19" s="20">
+        <v>233</v>
+      </c>
+      <c r="D19" s="20">
+        <v>479.46</v>
+      </c>
+      <c r="E19" s="20">
+        <v>34</v>
+      </c>
+      <c r="F19" s="21">
+        <v>5</v>
+      </c>
+      <c r="G19" s="9"/>
+      <c r="H19" s="9"/>
+      <c r="I19" s="9"/>
+      <c r="J19" s="9"/>
+      <c r="K19" s="9"/>
+      <c r="L19" s="9"/>
+    </row>
+    <row r="20" spans="1:12" ht="13.8" thickBot="1">
+      <c r="A20" s="24">
+        <v>6</v>
+      </c>
+      <c r="B20" s="25"/>
+      <c r="C20" s="20">
+        <v>298</v>
+      </c>
+      <c r="D20" s="20">
+        <v>631.97</v>
+      </c>
+      <c r="E20" s="20">
+        <v>42</v>
+      </c>
+      <c r="F20" s="21">
+        <v>6</v>
+      </c>
+      <c r="G20" s="9"/>
+      <c r="H20" s="9"/>
+      <c r="I20" s="9"/>
+      <c r="J20" s="9"/>
+      <c r="K20" s="9"/>
+      <c r="L20" s="9"/>
+    </row>
+    <row r="21" spans="1:12" ht="13.8" thickBot="1">
+      <c r="A21" s="25"/>
+      <c r="B21" s="24">
+        <v>7</v>
+      </c>
+      <c r="C21" s="20">
+        <v>358</v>
+      </c>
+      <c r="D21" s="20">
+        <v>783.38</v>
+      </c>
+      <c r="E21" s="20">
+        <v>49</v>
+      </c>
+      <c r="F21" s="21">
+        <v>7</v>
+      </c>
+      <c r="G21" s="9"/>
+      <c r="H21" s="9"/>
+      <c r="I21" s="9"/>
+      <c r="J21" s="9"/>
+      <c r="K21" s="9"/>
+      <c r="L21" s="9"/>
+    </row>
+    <row r="22" spans="1:12" ht="13.8" thickBot="1">
+      <c r="A22" s="24">
+        <v>8</v>
+      </c>
+      <c r="B22" s="25"/>
+      <c r="C22" s="20">
+        <v>417</v>
+      </c>
+      <c r="D22" s="20">
+        <v>937.91</v>
+      </c>
+      <c r="E22" s="20">
+        <v>56</v>
+      </c>
+      <c r="F22" s="21">
+        <v>8</v>
+      </c>
+      <c r="G22" s="9"/>
+      <c r="H22" s="9"/>
+      <c r="I22" s="9"/>
+      <c r="J22" s="9"/>
+      <c r="K22" s="9"/>
+      <c r="L22" s="9"/>
+    </row>
+    <row r="23" spans="1:12" ht="13.8" thickBot="1">
+      <c r="A23" s="25"/>
+      <c r="B23" s="24">
+        <v>9</v>
+      </c>
+      <c r="C23" s="20">
+        <v>476</v>
+      </c>
+      <c r="D23" s="20">
+        <v>1098.6199999999999</v>
+      </c>
+      <c r="E23" s="20">
+        <v>63</v>
+      </c>
+      <c r="F23" s="21">
+        <v>9</v>
+      </c>
+      <c r="G23" s="9"/>
+      <c r="H23" s="9"/>
+      <c r="I23" s="9"/>
+      <c r="J23" s="9"/>
+      <c r="K23" s="9"/>
+      <c r="L23" s="9"/>
+    </row>
+    <row r="24" spans="1:12" ht="13.8" thickBot="1">
+      <c r="A24" s="24">
+        <v>10</v>
+      </c>
+      <c r="B24" s="25"/>
+      <c r="C24" s="20">
+        <v>537</v>
+      </c>
+      <c r="D24" s="20">
+        <v>1265.47</v>
+      </c>
+      <c r="E24" s="20">
+        <v>70</v>
+      </c>
+      <c r="F24" s="21">
+        <v>10</v>
+      </c>
+      <c r="G24" s="9"/>
+      <c r="H24" s="9"/>
+      <c r="I24" s="9"/>
+      <c r="J24" s="9"/>
+      <c r="K24" s="9"/>
+      <c r="L24" s="9"/>
+    </row>
+    <row r="25" spans="1:12" ht="13.8" thickBot="1">
+      <c r="A25" s="25"/>
+      <c r="B25" s="24">
+        <v>11</v>
+      </c>
+      <c r="C25" s="20">
+        <v>603</v>
+      </c>
+      <c r="D25" s="20">
+        <v>1448.32</v>
+      </c>
+      <c r="E25" s="20">
+        <v>78</v>
+      </c>
+      <c r="F25" s="21">
+        <v>11</v>
+      </c>
+      <c r="G25" s="9"/>
+      <c r="H25" s="9"/>
+      <c r="I25" s="9"/>
+      <c r="J25" s="9"/>
+      <c r="K25" s="9"/>
+      <c r="L25" s="9"/>
+    </row>
+    <row r="26" spans="1:12" ht="13.8" thickBot="1">
+      <c r="A26" s="24">
+        <v>12</v>
+      </c>
+      <c r="B26" s="25"/>
+      <c r="C26" s="20">
+        <v>674</v>
+      </c>
+      <c r="D26" s="20">
+        <v>1648.27</v>
+      </c>
+      <c r="E26" s="20">
+        <v>86</v>
+      </c>
+      <c r="F26" s="21">
+        <v>12</v>
+      </c>
+      <c r="G26" s="9"/>
+      <c r="H26" s="9"/>
+      <c r="I26" s="9"/>
+      <c r="J26" s="9"/>
+      <c r="K26" s="9"/>
+      <c r="L26" s="9"/>
+    </row>
+    <row r="27" spans="1:12" ht="13.8" thickBot="1">
+      <c r="A27" s="25"/>
+      <c r="B27" s="24">
+        <v>13</v>
+      </c>
+      <c r="C27" s="20">
+        <v>753</v>
+      </c>
+      <c r="D27" s="20">
+        <v>1876.08</v>
+      </c>
+      <c r="E27" s="20">
+        <v>95</v>
+      </c>
+      <c r="F27" s="21">
+        <v>13</v>
+      </c>
+      <c r="G27" s="9"/>
+      <c r="H27" s="9"/>
+      <c r="I27" s="9"/>
+      <c r="J27" s="9"/>
+      <c r="K27" s="9"/>
+      <c r="L27" s="9"/>
+    </row>
+    <row r="28" spans="1:12" ht="13.8" thickBot="1">
+      <c r="A28" s="24">
+        <v>14</v>
+      </c>
+      <c r="B28" s="25"/>
+      <c r="C28" s="20">
+        <v>843</v>
+      </c>
+      <c r="D28" s="20">
+        <v>2142.06</v>
+      </c>
+      <c r="E28" s="20">
+        <v>105</v>
+      </c>
+      <c r="F28" s="21">
+        <v>14</v>
+      </c>
+      <c r="G28" s="9"/>
+      <c r="H28" s="9"/>
+      <c r="I28" s="9"/>
+      <c r="J28" s="9"/>
+      <c r="K28" s="9"/>
+      <c r="L28" s="9"/>
+    </row>
+    <row r="29" spans="1:12" ht="13.8" thickBot="1">
+      <c r="A29" s="25"/>
+      <c r="B29" s="24">
+        <v>15</v>
+      </c>
+      <c r="C29" s="20">
+        <v>949</v>
+      </c>
+      <c r="D29" s="20">
+        <v>2465.37</v>
+      </c>
+      <c r="E29" s="20">
+        <v>117</v>
+      </c>
+      <c r="F29" s="21">
+        <v>15</v>
+      </c>
+      <c r="G29" s="9"/>
+      <c r="H29" s="9"/>
+      <c r="I29" s="9"/>
+      <c r="J29" s="9"/>
+      <c r="K29" s="9"/>
+      <c r="L29" s="9"/>
+    </row>
+    <row r="30" spans="1:12" ht="13.8" thickBot="1">
+      <c r="A30" s="24">
+        <v>16</v>
+      </c>
+      <c r="B30" s="25"/>
+      <c r="C30" s="20">
+        <v>1076</v>
+      </c>
+      <c r="D30" s="20">
+        <v>2866.31</v>
+      </c>
+      <c r="E30" s="20">
+        <v>130</v>
+      </c>
+      <c r="F30" s="21">
+        <v>16</v>
+      </c>
+      <c r="G30" s="9"/>
+      <c r="H30" s="9"/>
+      <c r="I30" s="9"/>
+      <c r="J30" s="9"/>
+      <c r="K30" s="9"/>
+      <c r="L30" s="9"/>
+    </row>
+    <row r="31" spans="1:12" ht="13.8" thickBot="1">
+      <c r="A31" s="25"/>
+      <c r="B31" s="24">
+        <v>17</v>
+      </c>
+      <c r="C31" s="20">
+        <v>1237</v>
+      </c>
+      <c r="D31" s="20">
+        <v>3401.59</v>
+      </c>
+      <c r="E31" s="20">
+        <v>147</v>
+      </c>
+      <c r="F31" s="21">
+        <v>17</v>
+      </c>
+      <c r="G31" s="9"/>
+      <c r="H31" s="9"/>
+      <c r="I31" s="9"/>
+      <c r="J31" s="9"/>
+      <c r="K31" s="9"/>
+      <c r="L31" s="9"/>
+    </row>
+    <row r="32" spans="1:12" ht="13.8" thickBot="1">
+      <c r="A32" s="24">
+        <v>18</v>
+      </c>
+      <c r="B32" s="25"/>
+      <c r="C32" s="20">
+        <v>1459</v>
+      </c>
+      <c r="D32" s="20">
+        <v>4155.7299999999996</v>
+      </c>
+      <c r="E32" s="20">
+        <v>170</v>
+      </c>
+      <c r="F32" s="21">
+        <v>18</v>
+      </c>
+      <c r="G32" s="9"/>
+      <c r="H32" s="9"/>
+      <c r="I32" s="9"/>
+      <c r="J32" s="9"/>
+      <c r="K32" s="9"/>
+      <c r="L32" s="9"/>
+    </row>
+    <row r="33" spans="1:12" ht="13.8" thickBot="1">
+      <c r="A33" s="25"/>
+      <c r="B33" s="24">
+        <v>19</v>
+      </c>
+      <c r="C33" s="20">
+        <v>1801</v>
+      </c>
+      <c r="D33" s="20">
+        <v>5400.08</v>
+      </c>
+      <c r="E33" s="20">
+        <v>205</v>
+      </c>
+      <c r="F33" s="21">
+        <v>19</v>
+      </c>
+      <c r="G33" s="9"/>
+      <c r="H33" s="9"/>
+      <c r="I33" s="9"/>
+      <c r="J33" s="9"/>
+      <c r="K33" s="9"/>
+      <c r="L33" s="9"/>
+    </row>
+    <row r="34" spans="1:12" ht="13.8" thickBot="1">
+      <c r="A34" s="24">
+        <v>20</v>
+      </c>
+      <c r="B34" s="25"/>
+      <c r="C34" s="20">
+        <v>2479</v>
+      </c>
+      <c r="D34" s="20">
+        <v>8037.54</v>
+      </c>
+      <c r="E34" s="20">
+        <v>281</v>
+      </c>
+      <c r="F34" s="21">
+        <v>20</v>
+      </c>
+      <c r="G34" s="9"/>
+      <c r="H34" s="9"/>
+      <c r="I34" s="9"/>
+      <c r="J34" s="9"/>
+      <c r="K34" s="9"/>
+      <c r="L34" s="9"/>
+    </row>
+    <row r="35" spans="1:12" ht="13.8" thickBot="1">
+      <c r="A35" s="25"/>
+      <c r="B35" s="24">
+        <v>21</v>
+      </c>
+      <c r="C35" s="20">
+        <v>594601</v>
+      </c>
+      <c r="D35" s="20">
+        <v>223212</v>
+      </c>
+      <c r="E35" s="20">
+        <v>3920</v>
+      </c>
+      <c r="F35" s="21">
+        <v>21</v>
+      </c>
+      <c r="G35" s="9"/>
+      <c r="H35" s="9"/>
+      <c r="I35" s="9"/>
+      <c r="J35" s="9"/>
+      <c r="K35" s="9"/>
+      <c r="L35" s="9"/>
+    </row>
+    <row r="36" spans="1:12" ht="13.8" thickBot="1">
+      <c r="A36" s="19"/>
+      <c r="B36" s="25"/>
+      <c r="C36" s="22"/>
+      <c r="D36" s="22"/>
+      <c r="E36" s="22"/>
+      <c r="F36" s="23"/>
+      <c r="G36" s="9"/>
+      <c r="H36" s="9"/>
+      <c r="I36" s="9"/>
+      <c r="J36" s="9"/>
+      <c r="K36" s="9"/>
+      <c r="L36" s="9"/>
+    </row>
+  </sheetData>
+  <mergeCells count="22">
+    <mergeCell ref="A14:B14"/>
+    <mergeCell ref="B15:B16"/>
+    <mergeCell ref="A16:A17"/>
+    <mergeCell ref="B17:B18"/>
+    <mergeCell ref="A18:A19"/>
+    <mergeCell ref="B19:B20"/>
+    <mergeCell ref="A20:A21"/>
+    <mergeCell ref="B21:B22"/>
+    <mergeCell ref="A22:A23"/>
+    <mergeCell ref="B23:B24"/>
+    <mergeCell ref="A34:A35"/>
+    <mergeCell ref="B35:B36"/>
+    <mergeCell ref="A24:A25"/>
+    <mergeCell ref="B25:B26"/>
+    <mergeCell ref="A26:A27"/>
+    <mergeCell ref="B27:B28"/>
+    <mergeCell ref="A28:A29"/>
+    <mergeCell ref="B29:B30"/>
+    <mergeCell ref="A30:A31"/>
+    <mergeCell ref="B31:B32"/>
+    <mergeCell ref="A32:A33"/>
+    <mergeCell ref="B33:B34"/>
+  </mergeCells>
+  <hyperlinks>
+    <hyperlink ref="A9" r:id="rId1" display="http://nomdusite.com/" xr:uid="{A8AC6E5D-FD7B-4FC9-A0EA-11D6BDEE398B}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:AA23"/>

</xml_diff>